<commit_message>
Working on C_Y theory
</commit_message>
<xml_diff>
--- a/report_scripts/Matos Henrique/AggRegionCTheory/gha1971.xlsx
+++ b/report_scripts/Matos Henrique/AggRegionCTheory/gha1971.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mkh2/github/PFUPipeline2/report_scripts/Matos Henrique/AggRegionCTheory/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{086A6D83-DF1A-FA4B-94AE-3062D84C6B29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="44280" windowHeight="33960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="44280" windowHeight="33960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GHA-1971-E-Final" sheetId="2" r:id="rId1"/>
@@ -562,7 +562,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -579,18 +579,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1635,23 +1631,23 @@
       <c r="B17" s="5">
         <v>1</v>
       </c>
-      <c r="T17" s="6" t="s">
+      <c r="T17" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="U17" s="7"/>
-      <c r="V17" s="7"/>
-      <c r="W17" s="7"/>
-      <c r="X17" s="7"/>
-      <c r="AB17" s="6" t="s">
+      <c r="U17" s="9"/>
+      <c r="V17" s="9"/>
+      <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
+      <c r="AB17" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="AC17" s="7"/>
-      <c r="AD17" s="7"/>
-      <c r="AE17" s="7"/>
-      <c r="AF17" s="7"/>
+      <c r="AC17" s="9"/>
+      <c r="AD17" s="9"/>
+      <c r="AE17" s="9"/>
+      <c r="AF17" s="9"/>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="8" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1973,13 +1969,13 @@
       </c>
     </row>
     <row r="36" spans="19:47" x14ac:dyDescent="0.2">
-      <c r="T36" s="6" t="s">
+      <c r="T36" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="U36" s="7"/>
-      <c r="V36" s="7"/>
-      <c r="W36" s="7"/>
-      <c r="X36" s="7"/>
+      <c r="U36" s="9"/>
+      <c r="V36" s="9"/>
+      <c r="W36" s="9"/>
+      <c r="X36" s="9"/>
     </row>
     <row r="39" spans="19:47" ht="334" x14ac:dyDescent="0.2">
       <c r="T39" s="3" t="s">
@@ -3304,35 +3300,35 @@
       </c>
     </row>
     <row r="55" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="T55" s="6" t="s">
+      <c r="T55" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="U55" s="7"/>
-      <c r="V55" s="7"/>
-      <c r="W55" s="7"/>
-      <c r="X55" s="7"/>
-      <c r="AB55" s="6" t="s">
+      <c r="U55" s="9"/>
+      <c r="V55" s="9"/>
+      <c r="W55" s="9"/>
+      <c r="X55" s="9"/>
+      <c r="AB55" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="AC55" s="7"/>
-      <c r="AD55" s="7"/>
-      <c r="AE55" s="7"/>
-      <c r="AF55" s="7"/>
-      <c r="AG55" s="7"/>
-      <c r="AH55" s="7"/>
-      <c r="AI55" s="7"/>
-      <c r="AJ55" s="7"/>
-      <c r="AK55" s="7"/>
-      <c r="AL55" s="7"/>
-      <c r="AM55" s="7"/>
-      <c r="AN55" s="7"/>
-      <c r="AO55" s="7"/>
-      <c r="AP55" s="7"/>
-      <c r="AQ55" s="7"/>
-      <c r="AR55" s="7"/>
-      <c r="AS55" s="7"/>
-      <c r="AT55" s="7"/>
-      <c r="AU55" s="7"/>
+      <c r="AC55" s="9"/>
+      <c r="AD55" s="9"/>
+      <c r="AE55" s="9"/>
+      <c r="AF55" s="9"/>
+      <c r="AG55" s="9"/>
+      <c r="AH55" s="9"/>
+      <c r="AI55" s="9"/>
+      <c r="AJ55" s="9"/>
+      <c r="AK55" s="9"/>
+      <c r="AL55" s="9"/>
+      <c r="AM55" s="9"/>
+      <c r="AN55" s="9"/>
+      <c r="AO55" s="9"/>
+      <c r="AP55" s="9"/>
+      <c r="AQ55" s="9"/>
+      <c r="AR55" s="9"/>
+      <c r="AS55" s="9"/>
+      <c r="AT55" s="9"/>
+      <c r="AU55" s="9"/>
     </row>
     <row r="58" spans="1:47" ht="182" x14ac:dyDescent="0.2">
       <c r="B58" s="3" t="s">
@@ -3632,23 +3628,23 @@
       </c>
     </row>
     <row r="64" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="B64" s="6" t="s">
+      <c r="B64" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C64" s="7"/>
-      <c r="D64" s="7"/>
-      <c r="E64" s="7"/>
-      <c r="F64" s="7"/>
-      <c r="G64" s="7"/>
-      <c r="H64" s="7"/>
-      <c r="I64" s="7"/>
-      <c r="J64" s="7"/>
-      <c r="K64" s="7"/>
-      <c r="L64" s="7"/>
-      <c r="M64" s="7"/>
-      <c r="N64" s="7"/>
-      <c r="O64" s="7"/>
-      <c r="P64" s="7"/>
+      <c r="C64" s="9"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="9"/>
+      <c r="F64" s="9"/>
+      <c r="G64" s="9"/>
+      <c r="H64" s="9"/>
+      <c r="I64" s="9"/>
+      <c r="J64" s="9"/>
+      <c r="K64" s="9"/>
+      <c r="L64" s="9"/>
+      <c r="M64" s="9"/>
+      <c r="N64" s="9"/>
+      <c r="O64" s="9"/>
+      <c r="P64" s="9"/>
     </row>
     <row r="67" spans="1:16" ht="182" x14ac:dyDescent="0.2">
       <c r="B67" s="3" t="s">
@@ -4098,23 +4094,23 @@
       </c>
     </row>
     <row r="76" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B76" s="6" t="s">
+      <c r="B76" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C76" s="7"/>
-      <c r="D76" s="7"/>
-      <c r="E76" s="7"/>
-      <c r="F76" s="7"/>
-      <c r="G76" s="7"/>
-      <c r="H76" s="7"/>
-      <c r="I76" s="7"/>
-      <c r="J76" s="7"/>
-      <c r="K76" s="7"/>
-      <c r="L76" s="7"/>
-      <c r="M76" s="7"/>
-      <c r="N76" s="7"/>
-      <c r="O76" s="7"/>
-      <c r="P76" s="7"/>
+      <c r="C76" s="9"/>
+      <c r="D76" s="9"/>
+      <c r="E76" s="9"/>
+      <c r="F76" s="9"/>
+      <c r="G76" s="9"/>
+      <c r="H76" s="9"/>
+      <c r="I76" s="9"/>
+      <c r="J76" s="9"/>
+      <c r="K76" s="9"/>
+      <c r="L76" s="9"/>
+      <c r="M76" s="9"/>
+      <c r="N76" s="9"/>
+      <c r="O76" s="9"/>
+      <c r="P76" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -23295,113 +23291,113 @@
       <c r="B62" s="5">
         <v>0</v>
       </c>
-      <c r="BM62" s="6" t="s">
+      <c r="BM62" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="BN62" s="7"/>
-      <c r="BO62" s="7"/>
-      <c r="BP62" s="7"/>
-      <c r="BQ62" s="7"/>
-      <c r="BR62" s="7"/>
-      <c r="BS62" s="7"/>
-      <c r="BT62" s="7"/>
-      <c r="BU62" s="7"/>
-      <c r="BV62" s="7"/>
-      <c r="BW62" s="7"/>
-      <c r="BX62" s="7"/>
-      <c r="BY62" s="7"/>
-      <c r="BZ62" s="7"/>
-      <c r="CA62" s="7"/>
-      <c r="CB62" s="7"/>
-      <c r="CC62" s="7"/>
-      <c r="CD62" s="7"/>
-      <c r="CE62" s="7"/>
-      <c r="CF62" s="7"/>
-      <c r="CG62" s="7"/>
-      <c r="CH62" s="7"/>
-      <c r="CI62" s="7"/>
-      <c r="CJ62" s="7"/>
-      <c r="CK62" s="7"/>
-      <c r="CL62" s="7"/>
-      <c r="CM62" s="7"/>
-      <c r="CN62" s="7"/>
-      <c r="CO62" s="7"/>
-      <c r="CP62" s="7"/>
-      <c r="CQ62" s="7"/>
-      <c r="CR62" s="7"/>
-      <c r="CS62" s="7"/>
-      <c r="CT62" s="7"/>
-      <c r="CU62" s="7"/>
-      <c r="CV62" s="7"/>
-      <c r="CW62" s="7"/>
-      <c r="CX62" s="7"/>
-      <c r="CY62" s="7"/>
-      <c r="CZ62" s="7"/>
-      <c r="DA62" s="7"/>
-      <c r="DB62" s="7"/>
-      <c r="DC62" s="7"/>
-      <c r="DD62" s="7"/>
-      <c r="DE62" s="7"/>
-      <c r="DF62" s="7"/>
-      <c r="DG62" s="7"/>
-      <c r="DH62" s="7"/>
-      <c r="DI62" s="7"/>
-      <c r="DJ62" s="7"/>
-      <c r="DN62" s="6" t="s">
+      <c r="BN62" s="9"/>
+      <c r="BO62" s="9"/>
+      <c r="BP62" s="9"/>
+      <c r="BQ62" s="9"/>
+      <c r="BR62" s="9"/>
+      <c r="BS62" s="9"/>
+      <c r="BT62" s="9"/>
+      <c r="BU62" s="9"/>
+      <c r="BV62" s="9"/>
+      <c r="BW62" s="9"/>
+      <c r="BX62" s="9"/>
+      <c r="BY62" s="9"/>
+      <c r="BZ62" s="9"/>
+      <c r="CA62" s="9"/>
+      <c r="CB62" s="9"/>
+      <c r="CC62" s="9"/>
+      <c r="CD62" s="9"/>
+      <c r="CE62" s="9"/>
+      <c r="CF62" s="9"/>
+      <c r="CG62" s="9"/>
+      <c r="CH62" s="9"/>
+      <c r="CI62" s="9"/>
+      <c r="CJ62" s="9"/>
+      <c r="CK62" s="9"/>
+      <c r="CL62" s="9"/>
+      <c r="CM62" s="9"/>
+      <c r="CN62" s="9"/>
+      <c r="CO62" s="9"/>
+      <c r="CP62" s="9"/>
+      <c r="CQ62" s="9"/>
+      <c r="CR62" s="9"/>
+      <c r="CS62" s="9"/>
+      <c r="CT62" s="9"/>
+      <c r="CU62" s="9"/>
+      <c r="CV62" s="9"/>
+      <c r="CW62" s="9"/>
+      <c r="CX62" s="9"/>
+      <c r="CY62" s="9"/>
+      <c r="CZ62" s="9"/>
+      <c r="DA62" s="9"/>
+      <c r="DB62" s="9"/>
+      <c r="DC62" s="9"/>
+      <c r="DD62" s="9"/>
+      <c r="DE62" s="9"/>
+      <c r="DF62" s="9"/>
+      <c r="DG62" s="9"/>
+      <c r="DH62" s="9"/>
+      <c r="DI62" s="9"/>
+      <c r="DJ62" s="9"/>
+      <c r="DN62" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="DO62" s="7"/>
-      <c r="DP62" s="7"/>
-      <c r="DQ62" s="7"/>
-      <c r="DR62" s="7"/>
-      <c r="DS62" s="7"/>
-      <c r="DT62" s="7"/>
-      <c r="DU62" s="7"/>
-      <c r="DV62" s="7"/>
-      <c r="DW62" s="7"/>
-      <c r="DX62" s="7"/>
-      <c r="DY62" s="7"/>
-      <c r="DZ62" s="7"/>
-      <c r="EA62" s="7"/>
-      <c r="EB62" s="7"/>
-      <c r="EC62" s="7"/>
-      <c r="ED62" s="7"/>
-      <c r="EE62" s="7"/>
-      <c r="EF62" s="7"/>
-      <c r="EG62" s="7"/>
-      <c r="EH62" s="7"/>
-      <c r="EI62" s="7"/>
-      <c r="EJ62" s="7"/>
-      <c r="EK62" s="7"/>
-      <c r="EL62" s="7"/>
-      <c r="EM62" s="7"/>
-      <c r="EN62" s="7"/>
-      <c r="EO62" s="7"/>
-      <c r="EP62" s="7"/>
-      <c r="EQ62" s="7"/>
-      <c r="ER62" s="7"/>
-      <c r="ES62" s="7"/>
-      <c r="ET62" s="7"/>
-      <c r="EU62" s="7"/>
-      <c r="EV62" s="7"/>
-      <c r="EW62" s="7"/>
-      <c r="EX62" s="7"/>
-      <c r="EY62" s="7"/>
-      <c r="EZ62" s="7"/>
-      <c r="FA62" s="7"/>
-      <c r="FB62" s="7"/>
-      <c r="FC62" s="7"/>
-      <c r="FD62" s="7"/>
-      <c r="FE62" s="7"/>
-      <c r="FF62" s="7"/>
-      <c r="FG62" s="7"/>
-      <c r="FH62" s="7"/>
-      <c r="FI62" s="7"/>
-      <c r="FJ62" s="7"/>
-      <c r="FK62" s="7"/>
+      <c r="DO62" s="9"/>
+      <c r="DP62" s="9"/>
+      <c r="DQ62" s="9"/>
+      <c r="DR62" s="9"/>
+      <c r="DS62" s="9"/>
+      <c r="DT62" s="9"/>
+      <c r="DU62" s="9"/>
+      <c r="DV62" s="9"/>
+      <c r="DW62" s="9"/>
+      <c r="DX62" s="9"/>
+      <c r="DY62" s="9"/>
+      <c r="DZ62" s="9"/>
+      <c r="EA62" s="9"/>
+      <c r="EB62" s="9"/>
+      <c r="EC62" s="9"/>
+      <c r="ED62" s="9"/>
+      <c r="EE62" s="9"/>
+      <c r="EF62" s="9"/>
+      <c r="EG62" s="9"/>
+      <c r="EH62" s="9"/>
+      <c r="EI62" s="9"/>
+      <c r="EJ62" s="9"/>
+      <c r="EK62" s="9"/>
+      <c r="EL62" s="9"/>
+      <c r="EM62" s="9"/>
+      <c r="EN62" s="9"/>
+      <c r="EO62" s="9"/>
+      <c r="EP62" s="9"/>
+      <c r="EQ62" s="9"/>
+      <c r="ER62" s="9"/>
+      <c r="ES62" s="9"/>
+      <c r="ET62" s="9"/>
+      <c r="EU62" s="9"/>
+      <c r="EV62" s="9"/>
+      <c r="EW62" s="9"/>
+      <c r="EX62" s="9"/>
+      <c r="EY62" s="9"/>
+      <c r="EZ62" s="9"/>
+      <c r="FA62" s="9"/>
+      <c r="FB62" s="9"/>
+      <c r="FC62" s="9"/>
+      <c r="FD62" s="9"/>
+      <c r="FE62" s="9"/>
+      <c r="FF62" s="9"/>
+      <c r="FG62" s="9"/>
+      <c r="FH62" s="9"/>
+      <c r="FI62" s="9"/>
+      <c r="FJ62" s="9"/>
+      <c r="FK62" s="9"/>
     </row>
     <row r="63" spans="1:167" x14ac:dyDescent="0.2">
-      <c r="B63" s="6" t="s">
+      <c r="B63" s="8" t="s">
         <v>114</v>
       </c>
     </row>
@@ -32858,58 +32854,58 @@
       </c>
     </row>
     <row r="126" spans="64:114" x14ac:dyDescent="0.2">
-      <c r="BM126" s="6" t="s">
+      <c r="BM126" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="BN126" s="7"/>
-      <c r="BO126" s="7"/>
-      <c r="BP126" s="7"/>
-      <c r="BQ126" s="7"/>
-      <c r="BR126" s="7"/>
-      <c r="BS126" s="7"/>
-      <c r="BT126" s="7"/>
-      <c r="BU126" s="7"/>
-      <c r="BV126" s="7"/>
-      <c r="BW126" s="7"/>
-      <c r="BX126" s="7"/>
-      <c r="BY126" s="7"/>
-      <c r="BZ126" s="7"/>
-      <c r="CA126" s="7"/>
-      <c r="CB126" s="7"/>
-      <c r="CC126" s="7"/>
-      <c r="CD126" s="7"/>
-      <c r="CE126" s="7"/>
-      <c r="CF126" s="7"/>
-      <c r="CG126" s="7"/>
-      <c r="CH126" s="7"/>
-      <c r="CI126" s="7"/>
-      <c r="CJ126" s="7"/>
-      <c r="CK126" s="7"/>
-      <c r="CL126" s="7"/>
-      <c r="CM126" s="7"/>
-      <c r="CN126" s="7"/>
-      <c r="CO126" s="7"/>
-      <c r="CP126" s="7"/>
-      <c r="CQ126" s="7"/>
-      <c r="CR126" s="7"/>
-      <c r="CS126" s="7"/>
-      <c r="CT126" s="7"/>
-      <c r="CU126" s="7"/>
-      <c r="CV126" s="7"/>
-      <c r="CW126" s="7"/>
-      <c r="CX126" s="7"/>
-      <c r="CY126" s="7"/>
-      <c r="CZ126" s="7"/>
-      <c r="DA126" s="7"/>
-      <c r="DB126" s="7"/>
-      <c r="DC126" s="7"/>
-      <c r="DD126" s="7"/>
-      <c r="DE126" s="7"/>
-      <c r="DF126" s="7"/>
-      <c r="DG126" s="7"/>
-      <c r="DH126" s="7"/>
-      <c r="DI126" s="7"/>
-      <c r="DJ126" s="7"/>
+      <c r="BN126" s="9"/>
+      <c r="BO126" s="9"/>
+      <c r="BP126" s="9"/>
+      <c r="BQ126" s="9"/>
+      <c r="BR126" s="9"/>
+      <c r="BS126" s="9"/>
+      <c r="BT126" s="9"/>
+      <c r="BU126" s="9"/>
+      <c r="BV126" s="9"/>
+      <c r="BW126" s="9"/>
+      <c r="BX126" s="9"/>
+      <c r="BY126" s="9"/>
+      <c r="BZ126" s="9"/>
+      <c r="CA126" s="9"/>
+      <c r="CB126" s="9"/>
+      <c r="CC126" s="9"/>
+      <c r="CD126" s="9"/>
+      <c r="CE126" s="9"/>
+      <c r="CF126" s="9"/>
+      <c r="CG126" s="9"/>
+      <c r="CH126" s="9"/>
+      <c r="CI126" s="9"/>
+      <c r="CJ126" s="9"/>
+      <c r="CK126" s="9"/>
+      <c r="CL126" s="9"/>
+      <c r="CM126" s="9"/>
+      <c r="CN126" s="9"/>
+      <c r="CO126" s="9"/>
+      <c r="CP126" s="9"/>
+      <c r="CQ126" s="9"/>
+      <c r="CR126" s="9"/>
+      <c r="CS126" s="9"/>
+      <c r="CT126" s="9"/>
+      <c r="CU126" s="9"/>
+      <c r="CV126" s="9"/>
+      <c r="CW126" s="9"/>
+      <c r="CX126" s="9"/>
+      <c r="CY126" s="9"/>
+      <c r="CZ126" s="9"/>
+      <c r="DA126" s="9"/>
+      <c r="DB126" s="9"/>
+      <c r="DC126" s="9"/>
+      <c r="DD126" s="9"/>
+      <c r="DE126" s="9"/>
+      <c r="DF126" s="9"/>
+      <c r="DG126" s="9"/>
+      <c r="DH126" s="9"/>
+      <c r="DI126" s="9"/>
+      <c r="DJ126" s="9"/>
     </row>
     <row r="129" spans="64:137" ht="334" x14ac:dyDescent="0.2">
       <c r="BM129" s="3" t="s">
@@ -46204,80 +46200,80 @@
       </c>
     </row>
     <row r="190" spans="64:137" x14ac:dyDescent="0.2">
-      <c r="BM190" s="6" t="s">
+      <c r="BM190" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="BN190" s="7"/>
-      <c r="BO190" s="7"/>
-      <c r="BP190" s="7"/>
-      <c r="BQ190" s="7"/>
-      <c r="BR190" s="7"/>
-      <c r="BS190" s="7"/>
-      <c r="BT190" s="7"/>
-      <c r="BU190" s="7"/>
-      <c r="BV190" s="7"/>
-      <c r="BW190" s="7"/>
-      <c r="BX190" s="7"/>
-      <c r="BY190" s="7"/>
-      <c r="BZ190" s="7"/>
-      <c r="CA190" s="7"/>
-      <c r="CB190" s="7"/>
-      <c r="CC190" s="7"/>
-      <c r="CD190" s="7"/>
-      <c r="CE190" s="7"/>
-      <c r="CF190" s="7"/>
-      <c r="CG190" s="7"/>
-      <c r="CH190" s="7"/>
-      <c r="CI190" s="7"/>
-      <c r="CJ190" s="7"/>
-      <c r="CK190" s="7"/>
-      <c r="CL190" s="7"/>
-      <c r="CM190" s="7"/>
-      <c r="CN190" s="7"/>
-      <c r="CO190" s="7"/>
-      <c r="CP190" s="7"/>
-      <c r="CQ190" s="7"/>
-      <c r="CR190" s="7"/>
-      <c r="CS190" s="7"/>
-      <c r="CT190" s="7"/>
-      <c r="CU190" s="7"/>
-      <c r="CV190" s="7"/>
-      <c r="CW190" s="7"/>
-      <c r="CX190" s="7"/>
-      <c r="CY190" s="7"/>
-      <c r="CZ190" s="7"/>
-      <c r="DA190" s="7"/>
-      <c r="DB190" s="7"/>
-      <c r="DC190" s="7"/>
-      <c r="DD190" s="7"/>
-      <c r="DE190" s="7"/>
-      <c r="DF190" s="7"/>
-      <c r="DG190" s="7"/>
-      <c r="DH190" s="7"/>
-      <c r="DI190" s="7"/>
-      <c r="DJ190" s="7"/>
-      <c r="DN190" s="6" t="s">
+      <c r="BN190" s="9"/>
+      <c r="BO190" s="9"/>
+      <c r="BP190" s="9"/>
+      <c r="BQ190" s="9"/>
+      <c r="BR190" s="9"/>
+      <c r="BS190" s="9"/>
+      <c r="BT190" s="9"/>
+      <c r="BU190" s="9"/>
+      <c r="BV190" s="9"/>
+      <c r="BW190" s="9"/>
+      <c r="BX190" s="9"/>
+      <c r="BY190" s="9"/>
+      <c r="BZ190" s="9"/>
+      <c r="CA190" s="9"/>
+      <c r="CB190" s="9"/>
+      <c r="CC190" s="9"/>
+      <c r="CD190" s="9"/>
+      <c r="CE190" s="9"/>
+      <c r="CF190" s="9"/>
+      <c r="CG190" s="9"/>
+      <c r="CH190" s="9"/>
+      <c r="CI190" s="9"/>
+      <c r="CJ190" s="9"/>
+      <c r="CK190" s="9"/>
+      <c r="CL190" s="9"/>
+      <c r="CM190" s="9"/>
+      <c r="CN190" s="9"/>
+      <c r="CO190" s="9"/>
+      <c r="CP190" s="9"/>
+      <c r="CQ190" s="9"/>
+      <c r="CR190" s="9"/>
+      <c r="CS190" s="9"/>
+      <c r="CT190" s="9"/>
+      <c r="CU190" s="9"/>
+      <c r="CV190" s="9"/>
+      <c r="CW190" s="9"/>
+      <c r="CX190" s="9"/>
+      <c r="CY190" s="9"/>
+      <c r="CZ190" s="9"/>
+      <c r="DA190" s="9"/>
+      <c r="DB190" s="9"/>
+      <c r="DC190" s="9"/>
+      <c r="DD190" s="9"/>
+      <c r="DE190" s="9"/>
+      <c r="DF190" s="9"/>
+      <c r="DG190" s="9"/>
+      <c r="DH190" s="9"/>
+      <c r="DI190" s="9"/>
+      <c r="DJ190" s="9"/>
+      <c r="DN190" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="DO190" s="7"/>
-      <c r="DP190" s="7"/>
-      <c r="DQ190" s="7"/>
-      <c r="DR190" s="7"/>
-      <c r="DS190" s="7"/>
-      <c r="DT190" s="7"/>
-      <c r="DU190" s="7"/>
-      <c r="DV190" s="7"/>
-      <c r="DW190" s="7"/>
-      <c r="DX190" s="7"/>
-      <c r="DY190" s="7"/>
-      <c r="DZ190" s="7"/>
-      <c r="EA190" s="7"/>
-      <c r="EB190" s="7"/>
-      <c r="EC190" s="7"/>
-      <c r="ED190" s="7"/>
-      <c r="EE190" s="7"/>
-      <c r="EF190" s="7"/>
-      <c r="EG190" s="7"/>
+      <c r="DO190" s="9"/>
+      <c r="DP190" s="9"/>
+      <c r="DQ190" s="9"/>
+      <c r="DR190" s="9"/>
+      <c r="DS190" s="9"/>
+      <c r="DT190" s="9"/>
+      <c r="DU190" s="9"/>
+      <c r="DV190" s="9"/>
+      <c r="DW190" s="9"/>
+      <c r="DX190" s="9"/>
+      <c r="DY190" s="9"/>
+      <c r="DZ190" s="9"/>
+      <c r="EA190" s="9"/>
+      <c r="EB190" s="9"/>
+      <c r="EC190" s="9"/>
+      <c r="ED190" s="9"/>
+      <c r="EE190" s="9"/>
+      <c r="EF190" s="9"/>
+      <c r="EG190" s="9"/>
     </row>
     <row r="193" spans="1:61" ht="239" x14ac:dyDescent="0.2">
       <c r="B193" s="3" t="s">
@@ -55712,68 +55708,68 @@
       </c>
     </row>
     <row r="244" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="B244" s="6" t="s">
+      <c r="B244" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="C244" s="7"/>
-      <c r="D244" s="7"/>
-      <c r="E244" s="7"/>
-      <c r="F244" s="7"/>
-      <c r="G244" s="7"/>
-      <c r="H244" s="7"/>
-      <c r="I244" s="7"/>
-      <c r="J244" s="7"/>
-      <c r="K244" s="7"/>
-      <c r="L244" s="7"/>
-      <c r="M244" s="7"/>
-      <c r="N244" s="7"/>
-      <c r="O244" s="7"/>
-      <c r="P244" s="7"/>
-      <c r="Q244" s="7"/>
-      <c r="R244" s="7"/>
-      <c r="S244" s="7"/>
-      <c r="T244" s="7"/>
-      <c r="U244" s="7"/>
-      <c r="V244" s="7"/>
-      <c r="W244" s="7"/>
-      <c r="X244" s="7"/>
-      <c r="Y244" s="7"/>
-      <c r="Z244" s="7"/>
-      <c r="AA244" s="7"/>
-      <c r="AB244" s="7"/>
-      <c r="AC244" s="7"/>
-      <c r="AD244" s="7"/>
-      <c r="AE244" s="7"/>
-      <c r="AF244" s="7"/>
-      <c r="AG244" s="7"/>
-      <c r="AH244" s="7"/>
-      <c r="AI244" s="7"/>
-      <c r="AJ244" s="7"/>
-      <c r="AK244" s="7"/>
-      <c r="AL244" s="7"/>
-      <c r="AM244" s="7"/>
-      <c r="AN244" s="7"/>
-      <c r="AO244" s="7"/>
-      <c r="AP244" s="7"/>
-      <c r="AQ244" s="7"/>
-      <c r="AR244" s="7"/>
-      <c r="AS244" s="7"/>
-      <c r="AT244" s="7"/>
-      <c r="AU244" s="7"/>
-      <c r="AV244" s="7"/>
-      <c r="AW244" s="7"/>
-      <c r="AX244" s="7"/>
-      <c r="AY244" s="7"/>
-      <c r="AZ244" s="7"/>
-      <c r="BA244" s="7"/>
-      <c r="BB244" s="7"/>
-      <c r="BC244" s="7"/>
-      <c r="BD244" s="7"/>
-      <c r="BE244" s="7"/>
-      <c r="BF244" s="7"/>
-      <c r="BG244" s="7"/>
-      <c r="BH244" s="7"/>
-      <c r="BI244" s="7"/>
+      <c r="C244" s="9"/>
+      <c r="D244" s="9"/>
+      <c r="E244" s="9"/>
+      <c r="F244" s="9"/>
+      <c r="G244" s="9"/>
+      <c r="H244" s="9"/>
+      <c r="I244" s="9"/>
+      <c r="J244" s="9"/>
+      <c r="K244" s="9"/>
+      <c r="L244" s="9"/>
+      <c r="M244" s="9"/>
+      <c r="N244" s="9"/>
+      <c r="O244" s="9"/>
+      <c r="P244" s="9"/>
+      <c r="Q244" s="9"/>
+      <c r="R244" s="9"/>
+      <c r="S244" s="9"/>
+      <c r="T244" s="9"/>
+      <c r="U244" s="9"/>
+      <c r="V244" s="9"/>
+      <c r="W244" s="9"/>
+      <c r="X244" s="9"/>
+      <c r="Y244" s="9"/>
+      <c r="Z244" s="9"/>
+      <c r="AA244" s="9"/>
+      <c r="AB244" s="9"/>
+      <c r="AC244" s="9"/>
+      <c r="AD244" s="9"/>
+      <c r="AE244" s="9"/>
+      <c r="AF244" s="9"/>
+      <c r="AG244" s="9"/>
+      <c r="AH244" s="9"/>
+      <c r="AI244" s="9"/>
+      <c r="AJ244" s="9"/>
+      <c r="AK244" s="9"/>
+      <c r="AL244" s="9"/>
+      <c r="AM244" s="9"/>
+      <c r="AN244" s="9"/>
+      <c r="AO244" s="9"/>
+      <c r="AP244" s="9"/>
+      <c r="AQ244" s="9"/>
+      <c r="AR244" s="9"/>
+      <c r="AS244" s="9"/>
+      <c r="AT244" s="9"/>
+      <c r="AU244" s="9"/>
+      <c r="AV244" s="9"/>
+      <c r="AW244" s="9"/>
+      <c r="AX244" s="9"/>
+      <c r="AY244" s="9"/>
+      <c r="AZ244" s="9"/>
+      <c r="BA244" s="9"/>
+      <c r="BB244" s="9"/>
+      <c r="BC244" s="9"/>
+      <c r="BD244" s="9"/>
+      <c r="BE244" s="9"/>
+      <c r="BF244" s="9"/>
+      <c r="BG244" s="9"/>
+      <c r="BH244" s="9"/>
+      <c r="BI244" s="9"/>
     </row>
     <row r="247" spans="1:61" ht="239" x14ac:dyDescent="0.2">
       <c r="B247" s="3" t="s">
@@ -57438,68 +57434,68 @@
       </c>
     </row>
     <row r="256" spans="1:61" x14ac:dyDescent="0.2">
-      <c r="B256" s="6" t="s">
+      <c r="B256" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="C256" s="7"/>
-      <c r="D256" s="7"/>
-      <c r="E256" s="7"/>
-      <c r="F256" s="7"/>
-      <c r="G256" s="7"/>
-      <c r="H256" s="7"/>
-      <c r="I256" s="7"/>
-      <c r="J256" s="7"/>
-      <c r="K256" s="7"/>
-      <c r="L256" s="7"/>
-      <c r="M256" s="7"/>
-      <c r="N256" s="7"/>
-      <c r="O256" s="7"/>
-      <c r="P256" s="7"/>
-      <c r="Q256" s="7"/>
-      <c r="R256" s="7"/>
-      <c r="S256" s="7"/>
-      <c r="T256" s="7"/>
-      <c r="U256" s="7"/>
-      <c r="V256" s="7"/>
-      <c r="W256" s="7"/>
-      <c r="X256" s="7"/>
-      <c r="Y256" s="7"/>
-      <c r="Z256" s="7"/>
-      <c r="AA256" s="7"/>
-      <c r="AB256" s="7"/>
-      <c r="AC256" s="7"/>
-      <c r="AD256" s="7"/>
-      <c r="AE256" s="7"/>
-      <c r="AF256" s="7"/>
-      <c r="AG256" s="7"/>
-      <c r="AH256" s="7"/>
-      <c r="AI256" s="7"/>
-      <c r="AJ256" s="7"/>
-      <c r="AK256" s="7"/>
-      <c r="AL256" s="7"/>
-      <c r="AM256" s="7"/>
-      <c r="AN256" s="7"/>
-      <c r="AO256" s="7"/>
-      <c r="AP256" s="7"/>
-      <c r="AQ256" s="7"/>
-      <c r="AR256" s="7"/>
-      <c r="AS256" s="7"/>
-      <c r="AT256" s="7"/>
-      <c r="AU256" s="7"/>
-      <c r="AV256" s="7"/>
-      <c r="AW256" s="7"/>
-      <c r="AX256" s="7"/>
-      <c r="AY256" s="7"/>
-      <c r="AZ256" s="7"/>
-      <c r="BA256" s="7"/>
-      <c r="BB256" s="7"/>
-      <c r="BC256" s="7"/>
-      <c r="BD256" s="7"/>
-      <c r="BE256" s="7"/>
-      <c r="BF256" s="7"/>
-      <c r="BG256" s="7"/>
-      <c r="BH256" s="7"/>
-      <c r="BI256" s="7"/>
+      <c r="C256" s="9"/>
+      <c r="D256" s="9"/>
+      <c r="E256" s="9"/>
+      <c r="F256" s="9"/>
+      <c r="G256" s="9"/>
+      <c r="H256" s="9"/>
+      <c r="I256" s="9"/>
+      <c r="J256" s="9"/>
+      <c r="K256" s="9"/>
+      <c r="L256" s="9"/>
+      <c r="M256" s="9"/>
+      <c r="N256" s="9"/>
+      <c r="O256" s="9"/>
+      <c r="P256" s="9"/>
+      <c r="Q256" s="9"/>
+      <c r="R256" s="9"/>
+      <c r="S256" s="9"/>
+      <c r="T256" s="9"/>
+      <c r="U256" s="9"/>
+      <c r="V256" s="9"/>
+      <c r="W256" s="9"/>
+      <c r="X256" s="9"/>
+      <c r="Y256" s="9"/>
+      <c r="Z256" s="9"/>
+      <c r="AA256" s="9"/>
+      <c r="AB256" s="9"/>
+      <c r="AC256" s="9"/>
+      <c r="AD256" s="9"/>
+      <c r="AE256" s="9"/>
+      <c r="AF256" s="9"/>
+      <c r="AG256" s="9"/>
+      <c r="AH256" s="9"/>
+      <c r="AI256" s="9"/>
+      <c r="AJ256" s="9"/>
+      <c r="AK256" s="9"/>
+      <c r="AL256" s="9"/>
+      <c r="AM256" s="9"/>
+      <c r="AN256" s="9"/>
+      <c r="AO256" s="9"/>
+      <c r="AP256" s="9"/>
+      <c r="AQ256" s="9"/>
+      <c r="AR256" s="9"/>
+      <c r="AS256" s="9"/>
+      <c r="AT256" s="9"/>
+      <c r="AU256" s="9"/>
+      <c r="AV256" s="9"/>
+      <c r="AW256" s="9"/>
+      <c r="AX256" s="9"/>
+      <c r="AY256" s="9"/>
+      <c r="AZ256" s="9"/>
+      <c r="BA256" s="9"/>
+      <c r="BB256" s="9"/>
+      <c r="BC256" s="9"/>
+      <c r="BD256" s="9"/>
+      <c r="BE256" s="9"/>
+      <c r="BF256" s="9"/>
+      <c r="BG256" s="9"/>
+      <c r="BH256" s="9"/>
+      <c r="BI256" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -57554,7 +57550,7 @@
       <c r="N5" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="O5" s="11"/>
+      <c r="O5" s="3"/>
       <c r="AD5" s="3" t="s">
         <v>1</v>
       </c>
@@ -57740,7 +57736,7 @@
       <c r="N6" s="1">
         <v>0</v>
       </c>
-      <c r="O6" s="8"/>
+      <c r="O6" s="6"/>
       <c r="AC6" s="2" t="s">
         <v>51</v>
       </c>
@@ -57929,7 +57925,7 @@
       <c r="N7" s="1">
         <v>0</v>
       </c>
-      <c r="O7" s="8"/>
+      <c r="O7" s="6"/>
       <c r="AC7" s="2" t="s">
         <v>52</v>
       </c>
@@ -58118,7 +58114,7 @@
       <c r="N8" s="1">
         <v>0</v>
       </c>
-      <c r="O8" s="8"/>
+      <c r="O8" s="6"/>
       <c r="AC8" s="2" t="s">
         <v>53</v>
       </c>
@@ -58307,7 +58303,7 @@
       <c r="N9" s="1">
         <v>61.198500000000003</v>
       </c>
-      <c r="O9" s="8"/>
+      <c r="O9" s="6"/>
       <c r="AC9" s="2" t="s">
         <v>54</v>
       </c>
@@ -58496,7 +58492,7 @@
       <c r="N10" s="1">
         <v>0</v>
       </c>
-      <c r="O10" s="8"/>
+      <c r="O10" s="6"/>
       <c r="AC10" s="2" t="s">
         <v>55</v>
       </c>
@@ -58685,7 +58681,7 @@
       <c r="N11" s="1">
         <v>0</v>
       </c>
-      <c r="O11" s="8"/>
+      <c r="O11" s="6"/>
       <c r="AC11" s="2" t="s">
         <v>56</v>
       </c>
@@ -58874,7 +58870,7 @@
       <c r="N12" s="1">
         <v>0</v>
       </c>
-      <c r="O12" s="8"/>
+      <c r="O12" s="6"/>
       <c r="AC12" s="2" t="s">
         <v>57</v>
       </c>
@@ -59063,7 +59059,7 @@
       <c r="N13" s="1">
         <v>0</v>
       </c>
-      <c r="O13" s="8"/>
+      <c r="O13" s="6"/>
       <c r="AC13" s="2" t="s">
         <v>58</v>
       </c>
@@ -59252,7 +59248,7 @@
       <c r="N14" s="1">
         <v>0</v>
       </c>
-      <c r="O14" s="8"/>
+      <c r="O14" s="6"/>
       <c r="AC14" s="2" t="s">
         <v>59</v>
       </c>
@@ -59441,7 +59437,7 @@
       <c r="N15" s="1">
         <v>0</v>
       </c>
-      <c r="O15" s="8"/>
+      <c r="O15" s="6"/>
       <c r="AC15" s="2" t="s">
         <v>60</v>
       </c>
@@ -59630,7 +59626,7 @@
       <c r="N16" s="1">
         <v>0</v>
       </c>
-      <c r="O16" s="8"/>
+      <c r="O16" s="6"/>
       <c r="AC16" s="2" t="s">
         <v>61</v>
       </c>
@@ -59819,7 +59815,7 @@
       <c r="N17" s="1">
         <v>0</v>
       </c>
-      <c r="O17" s="8"/>
+      <c r="O17" s="6"/>
       <c r="AC17" s="2" t="s">
         <v>62</v>
       </c>
@@ -60008,7 +60004,7 @@
       <c r="N18" s="1">
         <v>0</v>
       </c>
-      <c r="O18" s="8"/>
+      <c r="O18" s="6"/>
       <c r="AC18" s="2" t="s">
         <v>63</v>
       </c>
@@ -60197,7 +60193,7 @@
       <c r="N19" s="1">
         <v>0</v>
       </c>
-      <c r="O19" s="8"/>
+      <c r="O19" s="6"/>
       <c r="AC19" s="2" t="s">
         <v>64</v>
       </c>
@@ -60386,7 +60382,7 @@
       <c r="N20" s="1">
         <v>0</v>
       </c>
-      <c r="O20" s="8"/>
+      <c r="O20" s="6"/>
       <c r="AC20" s="2" t="s">
         <v>65</v>
       </c>
@@ -60542,28 +60538,20 @@
       </c>
     </row>
     <row r="21" spans="4:79" x14ac:dyDescent="0.2">
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="F21" s="6"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="6"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="6"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="9"/>
-      <c r="Q21" s="10"/>
-      <c r="R21" s="10"/>
-      <c r="S21" s="10"/>
-      <c r="T21" s="10"/>
-      <c r="U21" s="10"/>
-      <c r="V21" s="10"/>
-      <c r="W21" s="10"/>
-      <c r="X21" s="10"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
       <c r="AC21" s="2" t="s">
         <v>66</v>
       </c>
@@ -64724,13 +64712,13 @@
       </c>
     </row>
     <row r="46" spans="4:79" x14ac:dyDescent="0.2">
-      <c r="E46" s="6" t="s">
+      <c r="E46" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="7"/>
-      <c r="I46" s="7"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="9"/>
       <c r="AC46" s="2" t="s">
         <v>92</v>
       </c>
@@ -67831,58 +67819,58 @@
       </c>
     </row>
     <row r="66" spans="29:79" x14ac:dyDescent="0.2">
-      <c r="AD66" s="6" t="s">
+      <c r="AD66" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="AE66" s="7"/>
-      <c r="AF66" s="7"/>
-      <c r="AG66" s="7"/>
-      <c r="AH66" s="7"/>
-      <c r="AI66" s="7"/>
-      <c r="AJ66" s="7"/>
-      <c r="AK66" s="7"/>
-      <c r="AL66" s="7"/>
-      <c r="AM66" s="7"/>
-      <c r="AN66" s="7"/>
-      <c r="AO66" s="7"/>
-      <c r="AP66" s="7"/>
-      <c r="AQ66" s="7"/>
-      <c r="AR66" s="7"/>
-      <c r="AS66" s="7"/>
-      <c r="AT66" s="7"/>
-      <c r="AU66" s="7"/>
-      <c r="AV66" s="7"/>
-      <c r="AW66" s="7"/>
-      <c r="AX66" s="7"/>
-      <c r="AY66" s="7"/>
-      <c r="AZ66" s="7"/>
-      <c r="BA66" s="7"/>
-      <c r="BB66" s="7"/>
-      <c r="BC66" s="7"/>
-      <c r="BD66" s="7"/>
-      <c r="BE66" s="7"/>
-      <c r="BF66" s="7"/>
-      <c r="BG66" s="7"/>
-      <c r="BH66" s="7"/>
-      <c r="BI66" s="7"/>
-      <c r="BJ66" s="7"/>
-      <c r="BK66" s="7"/>
-      <c r="BL66" s="7"/>
-      <c r="BM66" s="7"/>
-      <c r="BN66" s="7"/>
-      <c r="BO66" s="7"/>
-      <c r="BP66" s="7"/>
-      <c r="BQ66" s="7"/>
-      <c r="BR66" s="7"/>
-      <c r="BS66" s="7"/>
-      <c r="BT66" s="7"/>
-      <c r="BU66" s="7"/>
-      <c r="BV66" s="7"/>
-      <c r="BW66" s="7"/>
-      <c r="BX66" s="7"/>
-      <c r="BY66" s="7"/>
-      <c r="BZ66" s="7"/>
-      <c r="CA66" s="7"/>
+      <c r="AE66" s="9"/>
+      <c r="AF66" s="9"/>
+      <c r="AG66" s="9"/>
+      <c r="AH66" s="9"/>
+      <c r="AI66" s="9"/>
+      <c r="AJ66" s="9"/>
+      <c r="AK66" s="9"/>
+      <c r="AL66" s="9"/>
+      <c r="AM66" s="9"/>
+      <c r="AN66" s="9"/>
+      <c r="AO66" s="9"/>
+      <c r="AP66" s="9"/>
+      <c r="AQ66" s="9"/>
+      <c r="AR66" s="9"/>
+      <c r="AS66" s="9"/>
+      <c r="AT66" s="9"/>
+      <c r="AU66" s="9"/>
+      <c r="AV66" s="9"/>
+      <c r="AW66" s="9"/>
+      <c r="AX66" s="9"/>
+      <c r="AY66" s="9"/>
+      <c r="AZ66" s="9"/>
+      <c r="BA66" s="9"/>
+      <c r="BB66" s="9"/>
+      <c r="BC66" s="9"/>
+      <c r="BD66" s="9"/>
+      <c r="BE66" s="9"/>
+      <c r="BF66" s="9"/>
+      <c r="BG66" s="9"/>
+      <c r="BH66" s="9"/>
+      <c r="BI66" s="9"/>
+      <c r="BJ66" s="9"/>
+      <c r="BK66" s="9"/>
+      <c r="BL66" s="9"/>
+      <c r="BM66" s="9"/>
+      <c r="BN66" s="9"/>
+      <c r="BO66" s="9"/>
+      <c r="BP66" s="9"/>
+      <c r="BQ66" s="9"/>
+      <c r="BR66" s="9"/>
+      <c r="BS66" s="9"/>
+      <c r="BT66" s="9"/>
+      <c r="BU66" s="9"/>
+      <c r="BV66" s="9"/>
+      <c r="BW66" s="9"/>
+      <c r="BX66" s="9"/>
+      <c r="BY66" s="9"/>
+      <c r="BZ66" s="9"/>
+      <c r="CA66" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>